<commit_message>
feat(nfl): overhaul spread and total models with structural v5 engine, situational rest disparity, QB ratings, and divisional features
</commit_message>
<xml_diff>
--- a/data/sports/kbo/gated.xlsx
+++ b/data/sports/kbo/gated.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ104" headerRowCount="1">
-  <autoFilter ref="A1:DQ104"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ110" headerRowCount="1">
+  <autoFilter ref="A1:DQ110"/>
   <tableColumns count="121">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -780,19 +780,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$104)</f>
+        <f>COUNTA('Picks'!$A$2:$A$110)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$104,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$110,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$104,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$110,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"win")+COUNTIFS('Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"win")+COUNTIFS('Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -820,19 +820,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$104,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$110,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$104,"&gt;0",'Picks'!$V$2:$V$104,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$104,"&gt;0",'Picks'!$V$2:$V$104,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$110,"&gt;0",'Picks'!$V$2:$V$110,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$110,"&gt;0",'Picks'!$V$2:$V$110,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$104,"&gt;0",'Picks'!$V$2:$V$104,"win")/(COUNTIFS('Picks'!$BX$2:$BX$104,"&gt;0",'Picks'!$V$2:$V$104,"win")+COUNTIFS('Picks'!$BX$2:$BX$104,"&gt;0",'Picks'!$V$2:$V$104,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$110,"&gt;0",'Picks'!$V$2:$V$110,"win")/(COUNTIFS('Picks'!$BX$2:$BX$110,"&gt;0",'Picks'!$V$2:$V$110,"win")+COUNTIFS('Picks'!$BX$2:$BX$110,"&gt;0",'Picks'!$V$2:$V$110,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$104)/SUM('Picks'!$BX$2:$BX$104),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$110)/SUM('Picks'!$BX$2:$BX$110),0)</f>
         <v/>
       </c>
     </row>
@@ -860,19 +860,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$104)</f>
+        <f>SUM('Picks'!$BY$2:$BY$110)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$104,"&lt;&gt;",'Picks'!$AB$2:$AB$104),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$110,"&lt;&gt;",'Picks'!$AB$2:$AB$110),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$104,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$104,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$110,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$110,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$104,'Picks'!$AM$2:$AM$104,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$110,'Picks'!$AM$2:$AM$110,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -927,15 +927,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A14,'Picks'!$U$2:$U$104,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A14,'Picks'!$U$2:$U$110,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A14,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A14,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A14,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A14,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -943,11 +943,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$104,'Picks'!$H$2:$H$104,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$110,'Picks'!$H$2:$H$110,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$104,'Picks'!$H$2:$H$104,$A14,'Picks'!$U$2:$U$104,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$110,'Picks'!$H$2:$H$110,$A14,'Picks'!$U$2:$U$110,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -958,15 +958,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A15,'Picks'!$U$2:$U$104,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A15,'Picks'!$U$2:$U$110,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A15,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A15,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A15,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A15,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -974,11 +974,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$104,'Picks'!$H$2:$H$104,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$110,'Picks'!$H$2:$H$110,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$104,'Picks'!$H$2:$H$104,$A15,'Picks'!$U$2:$U$104,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$110,'Picks'!$H$2:$H$110,$A15,'Picks'!$U$2:$U$110,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -989,15 +989,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A16,'Picks'!$U$2:$U$104,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A16,'Picks'!$U$2:$U$110,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A16,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A16,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$104,$A16,'Picks'!$U$2:$U$104,"settled",'Picks'!$V$2:$V$104,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$110,$A16,'Picks'!$U$2:$U$110,"settled",'Picks'!$V$2:$V$110,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1005,11 +1005,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$104,'Picks'!$H$2:$H$104,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$110,'Picks'!$H$2:$H$110,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$104,'Picks'!$H$2:$H$104,$A16,'Picks'!$U$2:$U$104,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$110,'Picks'!$H$2:$H$110,$A16,'Picks'!$U$2:$U$110,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DQ104"/>
+  <dimension ref="A1:DQ110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -32836,12 +32836,12 @@
     <row r="100" ht="36" customHeight="1">
       <c r="A100" s="24" t="inlineStr">
         <is>
-          <t>3e71e6bc2182411b</t>
+          <t>62db88e1c5db4e23</t>
         </is>
       </c>
       <c r="B100" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="C100" s="24" t="inlineStr">
@@ -32886,23 +32886,23 @@
         </is>
       </c>
       <c r="L100" s="26" t="n">
-        <v>-122</v>
+        <v>-144</v>
       </c>
       <c r="M100" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.694444</v>
       </c>
       <c r="N100" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.590164</v>
       </c>
       <c r="O100" s="28" t="n">
         <v>0.581355</v>
       </c>
       <c r="P100" s="28" t="n"/>
       <c r="Q100" s="28" t="n">
-        <v>0.031805</v>
+        <v>-0.008809000000000001</v>
       </c>
       <c r="R100" s="26" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="S100" s="29" t="n">
         <v>1</v>
@@ -32914,21 +32914,41 @@
       </c>
       <c r="U100" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V100" s="24" t="n"/>
-      <c r="W100" s="26" t="n"/>
-      <c r="X100" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V100" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W100" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X100" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="Y100" s="25" t="n"/>
-      <c r="Z100" s="26" t="n"/>
-      <c r="AA100" s="28" t="n"/>
-      <c r="AB100" s="28" t="n"/>
-      <c r="AC100" s="30" t="n"/>
-      <c r="AD100" s="24" t="n"/>
+      <c r="Z100" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="AA100" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AB100" s="28" t="n">
+        <v>-0.010164</v>
+      </c>
+      <c r="AC100" s="30" t="n">
+        <v>0.6944</v>
+      </c>
+      <c r="AD100" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:06:37.779223Z</t>
+        </is>
+      </c>
       <c r="AE100" s="31" t="inlineStr">
         <is>
-          <t>Tie-aware Elo baseline; executable ask 0.5500 (market_slug=aec-kbo-sls-ndc-2026-10-07). Tie probability=0.0226.</t>
+          <t>Tie-aware Elo baseline; executable ask 0.5900 (market_slug=aec-kbo-sls-ndc-2026-10-07). Tie probability=0.0226.</t>
         </is>
       </c>
       <c r="AF100" s="31" t="inlineStr">
@@ -33012,7 +33032,7 @@
       </c>
       <c r="BA100" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BB100" s="24" t="inlineStr">
@@ -33027,7 +33047,7 @@
       </c>
       <c r="BD100" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BE100" s="24" t="inlineStr">
@@ -33047,7 +33067,7 @@
       </c>
       <c r="BH100" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:24:50.360101Z</t>
+          <t>2026-10-07T05:28:32.692035Z</t>
         </is>
       </c>
       <c r="BI100" s="24" t="inlineStr">
@@ -33057,19 +33077,23 @@
       </c>
       <c r="BJ100" s="25" t="n"/>
       <c r="BK100" s="26" t="n">
-        <v>-122</v>
+        <v>-144</v>
       </c>
       <c r="BL100" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.694444</v>
       </c>
       <c r="BM100" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.590164</v>
       </c>
       <c r="BN100" s="28" t="n"/>
       <c r="BO100" s="28" t="n"/>
       <c r="BP100" s="25" t="n"/>
-      <c r="BQ100" s="27" t="n"/>
-      <c r="BR100" s="28" t="n"/>
+      <c r="BQ100" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BR100" s="28" t="n">
+        <v>0.58</v>
+      </c>
       <c r="BS100" s="28" t="n"/>
       <c r="BT100" s="28" t="n"/>
       <c r="BU100" s="25" t="n"/>
@@ -33098,7 +33122,7 @@
       <c r="CR100" s="24" t="n"/>
       <c r="CS100" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="CT100" s="24" t="n"/>
@@ -33126,19 +33150,19 @@
       <c r="DP100" s="24" t="n"/>
       <c r="DQ100" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114", "away_team": "NC Dinos", "draw_settlement_value": 0.5, "event_id": "141706", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1470.713142, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1509.096592}, "historical_source_observation_times_verified": false, "home_team": "SSG Landers", "inference_inputs": {"away_id": "NC", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"NC": 1470.713142, "SSG": 1509.096592}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "f345eb917316d2e897f62c1cdd0f73153115c65da54c30c6137ad76bb7b27869"}, "home_id": "SSG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-06T22:24:50.283322+00:00", "outcome_probabilities": {"away": 0.40733144859905934, "draw": 0.02262693, "home": 0.5700416214009406}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.418645, "home": 0.581355}, "snapshot_hash": "31f08db0170bc67e3172ab16f112bf6397329449d8875dba363f80213cb3ec33", "sport": "KBO"}</t>
+          <t>{"artifact_hash": "72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a", "away_team": "NC Dinos", "draw_settlement_value": 0.5, "event_id": "141706", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1470.713142, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1509.096592}, "historical_source_observation_times_verified": false, "home_team": "SSG Landers", "inference_inputs": {"away_id": "NC", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"NC": 1470.713142, "SSG": 1509.096592}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "58ea522476e21dc70a719fe60647c19a772fcb4703fef8ed2d47c4ba7f07c2d5"}, "home_id": "SSG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-07T05:28:32.629666+00:00", "outcome_probabilities": {"away": 0.40733144859905934, "draw": 0.02262693, "home": 0.5700416214009406}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.418645, "home": 0.581355}, "snapshot_hash": "28dce38d0fc15f142228f9a356b5c6fdace64c9534c3a07f255be023a4118dfc", "sport": "KBO"}</t>
         </is>
       </c>
     </row>
     <row r="101" ht="36" customHeight="1">
       <c r="A101" s="24" t="inlineStr">
         <is>
-          <t>f9d68528eb0c4fce</t>
+          <t>111f561f9e784add</t>
         </is>
       </c>
       <c r="B101" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
@@ -33183,20 +33207,20 @@
         </is>
       </c>
       <c r="L101" s="26" t="n">
-        <v>-133</v>
+        <v>-127</v>
       </c>
       <c r="M101" s="27" t="n">
-        <v>1.75188</v>
+        <v>1.787402</v>
       </c>
       <c r="N101" s="28" t="n">
-        <v>0.570815</v>
+        <v>0.5594710000000001</v>
       </c>
       <c r="O101" s="28" t="n">
         <v>0.504038</v>
       </c>
       <c r="P101" s="28" t="n"/>
       <c r="Q101" s="28" t="n">
-        <v>-0.066777</v>
+        <v>-0.055433</v>
       </c>
       <c r="R101" s="26" t="n">
         <v>0</v>
@@ -33211,21 +33235,41 @@
       </c>
       <c r="U101" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V101" s="24" t="n"/>
-      <c r="W101" s="26" t="n"/>
-      <c r="X101" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V101" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W101" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X101" s="26" t="n">
+        <v>7</v>
+      </c>
       <c r="Y101" s="25" t="n"/>
-      <c r="Z101" s="26" t="n"/>
-      <c r="AA101" s="28" t="n"/>
-      <c r="AB101" s="28" t="n"/>
-      <c r="AC101" s="30" t="n"/>
-      <c r="AD101" s="24" t="n"/>
+      <c r="Z101" s="26" t="n">
+        <v>-127</v>
+      </c>
+      <c r="AA101" s="28" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB101" s="28" t="n">
+        <v>0.000529</v>
+      </c>
+      <c r="AC101" s="30" t="n">
+        <v>0.7874</v>
+      </c>
+      <c r="AD101" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:06:39.038081Z</t>
+        </is>
+      </c>
       <c r="AE101" s="31" t="inlineStr">
         <is>
-          <t>Tie-aware Elo baseline; executable ask 0.5700 (market_slug=aec-kbo-ltg-dbo-2026-10-07). Tie probability=0.0226.</t>
+          <t>Tie-aware Elo baseline; executable ask 0.5600 (market_slug=aec-kbo-ltg-dbo-2026-10-07). Tie probability=0.0226.</t>
         </is>
       </c>
       <c r="AF101" s="31" t="inlineStr">
@@ -33309,7 +33353,7 @@
       </c>
       <c r="BA101" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BB101" s="24" t="inlineStr">
@@ -33324,7 +33368,7 @@
       </c>
       <c r="BD101" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BE101" s="24" t="inlineStr">
@@ -33344,7 +33388,7 @@
       </c>
       <c r="BH101" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:24:50.421198Z</t>
+          <t>2026-10-07T05:28:32.757030Z</t>
         </is>
       </c>
       <c r="BI101" s="24" t="inlineStr">
@@ -33354,19 +33398,23 @@
       </c>
       <c r="BJ101" s="25" t="n"/>
       <c r="BK101" s="26" t="n">
-        <v>-133</v>
+        <v>-127</v>
       </c>
       <c r="BL101" s="27" t="n">
-        <v>1.75188</v>
+        <v>1.787402</v>
       </c>
       <c r="BM101" s="28" t="n">
-        <v>0.570815</v>
+        <v>0.5594710000000001</v>
       </c>
       <c r="BN101" s="28" t="n"/>
       <c r="BO101" s="28" t="n"/>
       <c r="BP101" s="25" t="n"/>
-      <c r="BQ101" s="27" t="n"/>
-      <c r="BR101" s="28" t="n"/>
+      <c r="BQ101" s="27" t="n">
+        <v>1.787402</v>
+      </c>
+      <c r="BR101" s="28" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="BS101" s="28" t="n"/>
       <c r="BT101" s="28" t="n"/>
       <c r="BU101" s="25" t="n"/>
@@ -33423,19 +33471,19 @@
       <c r="DP101" s="24" t="n"/>
       <c r="DQ101" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114", "away_team": "Doosan Bears", "draw_settlement_value": 0.5, "event_id": "141707", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1523.924017, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1506.794811}, "historical_source_observation_times_verified": false, "home_team": "LG Twins", "inference_inputs": {"away_id": "DOOSAN", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"DOOSAN": 1523.924017, "LG": 1506.794811}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "f345eb917316d2e897f62c1cdd0f73153115c65da54c30c6137ad76bb7b27869"}, "home_id": "LG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-06T22:24:50.283322+00:00", "outcome_probabilities": {"away": 0.484648703228405, "draw": 0.02262693, "home": 0.492724366771595}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.495962, "home": 0.504038}, "snapshot_hash": "cf1df3745177e4ea6b73c766e3bd90118f6d77b3d5d0fa9466d332ae291e5a03", "sport": "KBO"}</t>
+          <t>{"artifact_hash": "72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a", "away_team": "Doosan Bears", "draw_settlement_value": 0.5, "event_id": "141707", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1523.924017, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1506.794811}, "historical_source_observation_times_verified": false, "home_team": "LG Twins", "inference_inputs": {"away_id": "DOOSAN", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"DOOSAN": 1523.924017, "LG": 1506.794811}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "58ea522476e21dc70a719fe60647c19a772fcb4703fef8ed2d47c4ba7f07c2d5"}, "home_id": "LG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-07T05:28:32.629666+00:00", "outcome_probabilities": {"away": 0.484648703228405, "draw": 0.02262693, "home": 0.492724366771595}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.495962, "home": 0.504038}, "snapshot_hash": "afd033d4d28b8c64adf094a239b2036217e1f5a181bc3d411f635dc9a4692ef9", "sport": "KBO"}</t>
         </is>
       </c>
     </row>
     <row r="102" ht="36" customHeight="1">
       <c r="A102" s="24" t="inlineStr">
         <is>
-          <t>47c6aaba7be244be</t>
+          <t>8fe933b983b04274</t>
         </is>
       </c>
       <c r="B102" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="C102" s="24" t="inlineStr">
@@ -33480,23 +33528,23 @@
         </is>
       </c>
       <c r="L102" s="26" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="M102" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.961538</v>
       </c>
       <c r="N102" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.509804</v>
       </c>
       <c r="O102" s="28" t="n">
         <v>0.577223</v>
       </c>
       <c r="P102" s="28" t="n"/>
       <c r="Q102" s="28" t="n">
-        <v>0.057992</v>
+        <v>0.06741900000000001</v>
       </c>
       <c r="R102" s="26" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="S102" s="29" t="n">
         <v>1</v>
@@ -33508,21 +33556,41 @@
       </c>
       <c r="U102" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V102" s="24" t="n"/>
-      <c r="W102" s="26" t="n"/>
-      <c r="X102" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V102" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W102" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X102" s="26" t="n">
+        <v>9</v>
+      </c>
       <c r="Y102" s="25" t="n"/>
-      <c r="Z102" s="26" t="n"/>
-      <c r="AA102" s="28" t="n"/>
-      <c r="AB102" s="28" t="n"/>
-      <c r="AC102" s="30" t="n"/>
-      <c r="AD102" s="24" t="n"/>
+      <c r="Z102" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="AA102" s="28" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AB102" s="28" t="n">
+        <v>0.000196</v>
+      </c>
+      <c r="AC102" s="30" t="n">
+        <v>0.9615</v>
+      </c>
+      <c r="AD102" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:06:39.811929Z</t>
+        </is>
+      </c>
       <c r="AE102" s="31" t="inlineStr">
         <is>
-          <t>Tie-aware Elo baseline; executable ask 0.5200 (market_slug=aec-kbo-kwt-sla-2026-10-07). Tie probability=0.0226.</t>
+          <t>Tie-aware Elo baseline; executable ask 0.5100 (market_slug=aec-kbo-kwt-sla-2026-10-07). Tie probability=0.0226.</t>
         </is>
       </c>
       <c r="AF102" s="31" t="inlineStr">
@@ -33606,7 +33674,7 @@
       </c>
       <c r="BA102" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BB102" s="24" t="inlineStr">
@@ -33621,7 +33689,7 @@
       </c>
       <c r="BD102" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BE102" s="24" t="inlineStr">
@@ -33641,7 +33709,7 @@
       </c>
       <c r="BH102" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:24:50.489684Z</t>
+          <t>2026-10-07T05:28:32.894290Z</t>
         </is>
       </c>
       <c r="BI102" s="24" t="inlineStr">
@@ -33651,19 +33719,23 @@
       </c>
       <c r="BJ102" s="25" t="n"/>
       <c r="BK102" s="26" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="BL102" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.961538</v>
       </c>
       <c r="BM102" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.509804</v>
       </c>
       <c r="BN102" s="28" t="n"/>
       <c r="BO102" s="28" t="n"/>
       <c r="BP102" s="25" t="n"/>
-      <c r="BQ102" s="27" t="n"/>
-      <c r="BR102" s="28" t="n"/>
+      <c r="BQ102" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BR102" s="28" t="n">
+        <v>0.51</v>
+      </c>
       <c r="BS102" s="28" t="n"/>
       <c r="BT102" s="28" t="n"/>
       <c r="BU102" s="25" t="n"/>
@@ -33720,19 +33792,19 @@
       <c r="DP102" s="24" t="n"/>
       <c r="DQ102" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114", "away_team": "Samsung Lions", "draw_settlement_value": 0.5, "event_id": "141708", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1543.670103, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1579.036662}, "historical_source_observation_times_verified": false, "home_team": "KT Wiz", "inference_inputs": {"away_id": "SAMSUNG", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KT": 1579.036662, "SAMSUNG": 1543.670103}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "f345eb917316d2e897f62c1cdd0f73153115c65da54c30c6137ad76bb7b27869"}, "home_id": "KT", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-06T22:24:50.283322+00:00", "outcome_probabilities": {"away": 0.4114631296070524, "draw": 0.02262693, "home": 0.5659099403929476}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.422777, "home": 0.577223}, "snapshot_hash": "3fae4502ed3b14dbbf2cf166b4d67390c55d456648b342cdafced37495eacc0f", "sport": "KBO"}</t>
+          <t>{"artifact_hash": "72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a", "away_team": "Samsung Lions", "draw_settlement_value": 0.5, "event_id": "141708", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1543.670103, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1579.036662}, "historical_source_observation_times_verified": false, "home_team": "KT Wiz", "inference_inputs": {"away_id": "SAMSUNG", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KT": 1579.036662, "SAMSUNG": 1543.670103}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "58ea522476e21dc70a719fe60647c19a772fcb4703fef8ed2d47c4ba7f07c2d5"}, "home_id": "KT", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-07T05:28:32.629666+00:00", "outcome_probabilities": {"away": 0.4114631296070524, "draw": 0.02262693, "home": 0.5659099403929476}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.422777, "home": 0.577223}, "snapshot_hash": "d31379a8820d834cabbc3ee9cc08c7cb47f5e4af35d62037620e3185bc3ed430", "sport": "KBO"}</t>
         </is>
       </c>
     </row>
     <row r="103" ht="36" customHeight="1">
       <c r="A103" s="24" t="inlineStr">
         <is>
-          <t>8a6825759a1d472d</t>
+          <t>c9ba72464b35445c</t>
         </is>
       </c>
       <c r="B103" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="C103" s="24" t="inlineStr">
@@ -33777,20 +33849,20 @@
         </is>
       </c>
       <c r="L103" s="26" t="n">
-        <v>-163</v>
+        <v>-186</v>
       </c>
       <c r="M103" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.537634</v>
       </c>
       <c r="N103" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.65035</v>
       </c>
       <c r="O103" s="28" t="n">
         <v>0.5302480000000001</v>
       </c>
       <c r="P103" s="28" t="n"/>
       <c r="Q103" s="28" t="n">
-        <v>-0.08952400000000001</v>
+        <v>-0.120102</v>
       </c>
       <c r="R103" s="26" t="n">
         <v>0</v>
@@ -33805,21 +33877,41 @@
       </c>
       <c r="U103" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V103" s="24" t="n"/>
-      <c r="W103" s="26" t="n"/>
-      <c r="X103" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V103" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W103" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="X103" s="26" t="n">
+        <v>4</v>
+      </c>
       <c r="Y103" s="25" t="n"/>
-      <c r="Z103" s="26" t="n"/>
-      <c r="AA103" s="28" t="n"/>
-      <c r="AB103" s="28" t="n"/>
-      <c r="AC103" s="30" t="n"/>
-      <c r="AD103" s="24" t="n"/>
+      <c r="Z103" s="26" t="n">
+        <v>-186</v>
+      </c>
+      <c r="AA103" s="28" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AB103" s="28" t="n">
+        <v>-0.00035</v>
+      </c>
+      <c r="AC103" s="30" t="n">
+        <v>0.5376</v>
+      </c>
+      <c r="AD103" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:06:40.613506Z</t>
+        </is>
+      </c>
       <c r="AE103" s="31" t="inlineStr">
         <is>
-          <t>Tie-aware Elo baseline; executable ask 0.6200 (market_slug=aec-kbo-lgo-kti-2026-10-07). Tie probability=0.0226.</t>
+          <t>Tie-aware Elo baseline; executable ask 0.6500 (market_slug=aec-kbo-lgo-kti-2026-10-07). Tie probability=0.0226.</t>
         </is>
       </c>
       <c r="AF103" s="31" t="inlineStr">
@@ -33903,7 +33995,7 @@
       </c>
       <c r="BA103" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BB103" s="24" t="inlineStr">
@@ -33918,7 +34010,7 @@
       </c>
       <c r="BD103" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BE103" s="24" t="inlineStr">
@@ -33938,7 +34030,7 @@
       </c>
       <c r="BH103" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:24:50.570264Z</t>
+          <t>2026-10-07T05:28:32.949702Z</t>
         </is>
       </c>
       <c r="BI103" s="24" t="inlineStr">
@@ -33948,19 +34040,23 @@
       </c>
       <c r="BJ103" s="25" t="n"/>
       <c r="BK103" s="26" t="n">
-        <v>-163</v>
+        <v>-186</v>
       </c>
       <c r="BL103" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.537634</v>
       </c>
       <c r="BM103" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.65035</v>
       </c>
       <c r="BN103" s="28" t="n"/>
       <c r="BO103" s="28" t="n"/>
       <c r="BP103" s="25" t="n"/>
-      <c r="BQ103" s="27" t="n"/>
-      <c r="BR103" s="28" t="n"/>
+      <c r="BQ103" s="27" t="n">
+        <v>1.537634</v>
+      </c>
+      <c r="BR103" s="28" t="n">
+        <v>0.65</v>
+      </c>
       <c r="BS103" s="28" t="n"/>
       <c r="BT103" s="28" t="n"/>
       <c r="BU103" s="25" t="n"/>
@@ -34017,19 +34113,19 @@
       <c r="DP103" s="24" t="n"/>
       <c r="DQ103" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114", "away_team": "Kia Tigers", "draw_settlement_value": 0.5, "event_id": "141709", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1524.366838, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1482.834576}, "historical_source_observation_times_verified": false, "home_team": "Lotte Giants", "inference_inputs": {"away_id": "KIA", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KIA": 1524.366838, "LOTTE": 1482.834576}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "f345eb917316d2e897f62c1cdd0f73153115c65da54c30c6137ad76bb7b27869"}, "home_id": "LOTTE", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-06T22:24:50.283322+00:00", "outcome_probabilities": {"away": 0.5189340850239297, "draw": 0.02262693, "home": 0.4584389849760702}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.530248, "home": 0.469752}, "snapshot_hash": "7224fd777d486ed64d33b68c30084e68ac7193ae5a6ee397c4e0e18c916f3b21", "sport": "KBO"}</t>
+          <t>{"artifact_hash": "72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a", "away_team": "Kia Tigers", "draw_settlement_value": 0.5, "event_id": "141709", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1524.366838, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1482.834576}, "historical_source_observation_times_verified": false, "home_team": "Lotte Giants", "inference_inputs": {"away_id": "KIA", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KIA": 1524.366838, "LOTTE": 1482.834576}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "58ea522476e21dc70a719fe60647c19a772fcb4703fef8ed2d47c4ba7f07c2d5"}, "home_id": "LOTTE", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-07T05:28:32.629666+00:00", "outcome_probabilities": {"away": 0.5189340850239297, "draw": 0.02262693, "home": 0.4584389849760702}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.530248, "home": 0.469752}, "snapshot_hash": "048e2961bfb8400774b98a93c17330cd95e94c3aa95b43edaf021a161f941186", "sport": "KBO"}</t>
         </is>
       </c>
     </row>
     <row r="104" ht="36" customHeight="1">
       <c r="A104" s="24" t="inlineStr">
         <is>
-          <t>2a54ed97cd484cca</t>
+          <t>af66ba202d2d4c9c</t>
         </is>
       </c>
       <c r="B104" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="C104" s="24" t="inlineStr">
@@ -34102,18 +34198,38 @@
       </c>
       <c r="U104" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V104" s="24" t="n"/>
-      <c r="W104" s="26" t="n"/>
-      <c r="X104" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V104" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W104" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="X104" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="Y104" s="25" t="n"/>
-      <c r="Z104" s="26" t="n"/>
-      <c r="AA104" s="28" t="n"/>
-      <c r="AB104" s="28" t="n"/>
-      <c r="AC104" s="30" t="n"/>
-      <c r="AD104" s="24" t="n"/>
+      <c r="Z104" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="AA104" s="28" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AB104" s="28" t="n">
+        <v>0.000164</v>
+      </c>
+      <c r="AC104" s="30" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="AD104" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:06:41.351115Z</t>
+        </is>
+      </c>
       <c r="AE104" s="31" t="inlineStr">
         <is>
           <t>Tie-aware Elo baseline; executable ask 0.4100 (market_slug=aec-kbo-khi-hea-2026-10-07). Tie probability=0.0226.</t>
@@ -34200,7 +34316,7 @@
       </c>
       <c r="BA104" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BB104" s="24" t="inlineStr">
@@ -34215,7 +34331,7 @@
       </c>
       <c r="BD104" s="24" t="inlineStr">
         <is>
-          <t>7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114</t>
+          <t>72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a</t>
         </is>
       </c>
       <c r="BE104" s="24" t="inlineStr">
@@ -34235,7 +34351,7 @@
       </c>
       <c r="BH104" s="24" t="inlineStr">
         <is>
-          <t>2026-10-06T22:25:10.987601Z</t>
+          <t>2026-10-07T05:28:43.252505Z</t>
         </is>
       </c>
       <c r="BI104" s="24" t="inlineStr">
@@ -34256,8 +34372,12 @@
       <c r="BN104" s="28" t="n"/>
       <c r="BO104" s="28" t="n"/>
       <c r="BP104" s="25" t="n"/>
-      <c r="BQ104" s="27" t="n"/>
-      <c r="BR104" s="28" t="n"/>
+      <c r="BQ104" s="27" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="BR104" s="28" t="n">
+        <v>0.41</v>
+      </c>
       <c r="BS104" s="28" t="n"/>
       <c r="BT104" s="28" t="n"/>
       <c r="BU104" s="25" t="n"/>
@@ -34314,7 +34434,1889 @@
       <c r="DP104" s="24" t="n"/>
       <c r="DQ104" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "7cff2807fc660517fbda95f730a6a901b570d0845019c5e524dde23a826f7114", "away_team": "Hanwha Eagles", "draw_settlement_value": 0.5, "event_id": "141710", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1438.436026, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1440.024074}, "historical_source_observation_times_verified": false, "home_team": "Kiwoom Heroes", "inference_inputs": {"away_id": "HANWHA", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"HANWHA": 1438.436026, "KIWOOM": 1440.024074}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "f345eb917316d2e897f62c1cdd0f73153115c65da54c30c6137ad76bb7b27869"}, "home_id": "KIWOOM", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-06T22:24:50.283322+00:00", "outcome_probabilities": {"away": 0.45836082040103526, "draw": 0.02262693, "home": 0.5190122495989647}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.469674, "home": 0.530326}, "snapshot_hash": "322b7cf15492d4f871004a8d048c4176fc52dec89f029ce76c72682e2d17a07b", "sport": "KBO"}</t>
+          <t>{"artifact_hash": "72d934bf14f15b6340db5d573213dae372bfc880b7d95295d2b9d3795bdd3a0a", "away_team": "Hanwha Eagles", "draw_settlement_value": 0.5, "event_id": "141710", "event_start_utc": "2026-10-07T09:30:00Z", "features": {"away_elo": 1438.436026, "base_tie_rate": 0.02262693, "home_advantage": 20.0, "home_elo": 1440.024074}, "historical_source_observation_times_verified": false, "home_team": "Kiwoom Heroes", "inference_inputs": {"away_id": "HANWHA", "base_tie_rate": 0.02262693, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"HANWHA": 1438.436026, "KIWOOM": 1440.024074}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "58ea522476e21dc70a719fe60647c19a772fcb4703fef8ed2d47c4ba7f07c2d5"}, "home_id": "KIWOOM", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-07T05:28:32.629666+00:00", "outcome_probabilities": {"away": 0.45836082040103526, "draw": 0.02262693, "home": 0.5190122495989647}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.469674, "home": 0.530326}, "snapshot_hash": "907388d3fdba88097c0528b56a903f4aaac0dc5a91b17d6048a51098a120d5aa", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="36" customHeight="1">
+      <c r="A105" s="24" t="inlineStr">
+        <is>
+          <t>2a0342919749451f</t>
+        </is>
+      </c>
+      <c r="B105" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:06:46.442216Z</t>
+        </is>
+      </c>
+      <c r="C105" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T05:00:00Z</t>
+        </is>
+      </c>
+      <c r="D105" s="24" t="inlineStr">
+        <is>
+          <t>148641</t>
+        </is>
+      </c>
+      <c r="E105" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F105" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="G105" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="H105" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I105" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J105" s="25" t="n"/>
+      <c r="K105" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L105" s="26" t="n">
+        <v>-317</v>
+      </c>
+      <c r="M105" s="27" t="n">
+        <v>1.315457</v>
+      </c>
+      <c r="N105" s="28" t="n">
+        <v>0.760192</v>
+      </c>
+      <c r="O105" s="28" t="n">
+        <v>0.604778</v>
+      </c>
+      <c r="P105" s="28" t="n"/>
+      <c r="Q105" s="28" t="n">
+        <v>-0.155414</v>
+      </c>
+      <c r="R105" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T105" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U105" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V105" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W105" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="X105" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y105" s="25" t="n"/>
+      <c r="Z105" s="26" t="n"/>
+      <c r="AA105" s="28" t="n"/>
+      <c r="AB105" s="28" t="n"/>
+      <c r="AC105" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD105" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T10:04:04.404935Z</t>
+        </is>
+      </c>
+      <c r="AE105" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.7600 (market_slug=aec-kbo-kti-lgo-2026-10-11). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF105" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG105" s="24" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+      <c r="AH105" s="24" t="n"/>
+      <c r="AI105" s="31" t="n"/>
+      <c r="AJ105" s="31" t="n"/>
+      <c r="AK105" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL105" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM105" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN105" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO105" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP105" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AQ105" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AR105" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AS105" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AT105" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AU105" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AV105" s="24" t="n"/>
+      <c r="AW105" s="24" t="n"/>
+      <c r="AX105" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY105" s="24" t="n"/>
+      <c r="AZ105" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA105" s="24" t="inlineStr">
+        <is>
+          <t>341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb</t>
+        </is>
+      </c>
+      <c r="BB105" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC105" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD105" s="24" t="inlineStr">
+        <is>
+          <t>341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb</t>
+        </is>
+      </c>
+      <c r="BE105" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF105" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG105" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH105" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:06:46.388523Z</t>
+        </is>
+      </c>
+      <c r="BI105" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ105" s="25" t="n"/>
+      <c r="BK105" s="26" t="n">
+        <v>-317</v>
+      </c>
+      <c r="BL105" s="27" t="n">
+        <v>1.315457</v>
+      </c>
+      <c r="BM105" s="28" t="n">
+        <v>0.760192</v>
+      </c>
+      <c r="BN105" s="28" t="n"/>
+      <c r="BO105" s="28" t="n"/>
+      <c r="BP105" s="25" t="n"/>
+      <c r="BQ105" s="27" t="n"/>
+      <c r="BR105" s="28" t="n"/>
+      <c r="BS105" s="28" t="n"/>
+      <c r="BT105" s="28" t="n"/>
+      <c r="BU105" s="25" t="n"/>
+      <c r="BV105" s="29" t="n"/>
+      <c r="BW105" s="24" t="n"/>
+      <c r="BX105" s="30" t="n"/>
+      <c r="BY105" s="27" t="n"/>
+      <c r="BZ105" s="24" t="n"/>
+      <c r="CA105" s="31" t="n"/>
+      <c r="CB105" s="24" t="n"/>
+      <c r="CC105" s="24" t="n"/>
+      <c r="CD105" s="24" t="n"/>
+      <c r="CE105" s="24" t="n"/>
+      <c r="CF105" s="24" t="n"/>
+      <c r="CG105" s="24" t="n"/>
+      <c r="CH105" s="24" t="n"/>
+      <c r="CI105" s="24" t="n"/>
+      <c r="CJ105" s="24" t="n"/>
+      <c r="CK105" s="24" t="n"/>
+      <c r="CL105" s="24" t="n"/>
+      <c r="CM105" s="24" t="n"/>
+      <c r="CN105" s="24" t="n"/>
+      <c r="CO105" s="24" t="n"/>
+      <c r="CP105" s="24" t="n"/>
+      <c r="CQ105" s="24" t="n"/>
+      <c r="CR105" s="24" t="n"/>
+      <c r="CS105" s="24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="CT105" s="24" t="n"/>
+      <c r="CU105" s="24" t="n"/>
+      <c r="CV105" s="24" t="n"/>
+      <c r="CW105" s="24" t="n"/>
+      <c r="CX105" s="24" t="n"/>
+      <c r="CY105" s="24" t="n"/>
+      <c r="CZ105" s="24" t="n"/>
+      <c r="DA105" s="24" t="n"/>
+      <c r="DB105" s="24" t="n"/>
+      <c r="DC105" s="24" t="n"/>
+      <c r="DD105" s="24" t="n"/>
+      <c r="DE105" s="24" t="n"/>
+      <c r="DF105" s="24" t="n"/>
+      <c r="DG105" s="24" t="n"/>
+      <c r="DH105" s="24" t="n"/>
+      <c r="DI105" s="24" t="n"/>
+      <c r="DJ105" s="24" t="n"/>
+      <c r="DK105" s="24" t="n"/>
+      <c r="DL105" s="24" t="n"/>
+      <c r="DM105" s="24" t="n"/>
+      <c r="DN105" s="24" t="n"/>
+      <c r="DO105" s="24" t="n"/>
+      <c r="DP105" s="24" t="n"/>
+      <c r="DQ105" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb", "away_team": "Lotte Giants", "draw_settlement_value": 0.5, "event_id": "148641", "event_start_utc": "2026-10-11T05:00:00Z", "features": {"away_elo": 1479.387378, "base_tie_rate": 0.02259264, "home_advantage": 20.0, "home_elo": 1535.051436}, "historical_source_observation_times_verified": false, "home_team": "Kia Tigers", "inference_inputs": {"away_id": "LOTTE", "base_tie_rate": 0.02259264, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KIA": 1535.051436, "LOTTE": 1479.387378}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "KIA", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-11T01:06:46.324600+00:00", "outcome_probabilities": {"away": 0.3839256854980043, "draw": 0.02259264, "home": 0.5934816745019956}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.395222, "home": 0.604778}, "snapshot_hash": "93d5a7b26981d45a45f7121e46f9bc0accb1d8404bcafa61f4e38d5b72595fb1", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="36" customHeight="1">
+      <c r="A106" s="24" t="inlineStr">
+        <is>
+          <t>0de0c1d511de4f78</t>
+        </is>
+      </c>
+      <c r="B106" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:06:46.442216Z</t>
+        </is>
+      </c>
+      <c r="C106" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T05:00:00Z</t>
+        </is>
+      </c>
+      <c r="D106" s="24" t="inlineStr">
+        <is>
+          <t>148642</t>
+        </is>
+      </c>
+      <c r="E106" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F106" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="G106" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="H106" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I106" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J106" s="25" t="n"/>
+      <c r="K106" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L106" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M106" s="27" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="N106" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="O106" s="28" t="n">
+        <v>0.5353</v>
+      </c>
+      <c r="P106" s="28" t="n"/>
+      <c r="Q106" s="28" t="n">
+        <v>-0.003871</v>
+      </c>
+      <c r="R106" s="26" t="n">
+        <v>18</v>
+      </c>
+      <c r="S106" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T106" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U106" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V106" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W106" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="X106" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y106" s="25" t="n"/>
+      <c r="Z106" s="26" t="n"/>
+      <c r="AA106" s="28" t="n"/>
+      <c r="AB106" s="28" t="n"/>
+      <c r="AC106" s="30" t="n">
+        <v>0.8547</v>
+      </c>
+      <c r="AD106" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T10:04:05.573754Z</t>
+        </is>
+      </c>
+      <c r="AE106" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.5400 (market_slug=aec-kbo-sla-kwt-2026-10-11). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF106" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG106" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH106" s="24" t="n"/>
+      <c r="AI106" s="31" t="n"/>
+      <c r="AJ106" s="31" t="n"/>
+      <c r="AK106" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL106" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM106" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN106" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO106" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP106" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AQ106" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AR106" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AS106" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AT106" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AU106" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AV106" s="24" t="n"/>
+      <c r="AW106" s="24" t="n"/>
+      <c r="AX106" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY106" s="24" t="n"/>
+      <c r="AZ106" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA106" s="24" t="inlineStr">
+        <is>
+          <t>341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb</t>
+        </is>
+      </c>
+      <c r="BB106" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC106" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD106" s="24" t="inlineStr">
+        <is>
+          <t>341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb</t>
+        </is>
+      </c>
+      <c r="BE106" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF106" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG106" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH106" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:06:46.442216Z</t>
+        </is>
+      </c>
+      <c r="BI106" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ106" s="25" t="n"/>
+      <c r="BK106" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="BL106" s="27" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="BM106" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="BN106" s="28" t="n"/>
+      <c r="BO106" s="28" t="n"/>
+      <c r="BP106" s="25" t="n"/>
+      <c r="BQ106" s="27" t="n"/>
+      <c r="BR106" s="28" t="n"/>
+      <c r="BS106" s="28" t="n"/>
+      <c r="BT106" s="28" t="n"/>
+      <c r="BU106" s="25" t="n"/>
+      <c r="BV106" s="29" t="n"/>
+      <c r="BW106" s="24" t="n"/>
+      <c r="BX106" s="30" t="n"/>
+      <c r="BY106" s="27" t="n"/>
+      <c r="BZ106" s="24" t="n"/>
+      <c r="CA106" s="31" t="n"/>
+      <c r="CB106" s="24" t="n"/>
+      <c r="CC106" s="24" t="n"/>
+      <c r="CD106" s="24" t="n"/>
+      <c r="CE106" s="24" t="n"/>
+      <c r="CF106" s="24" t="n"/>
+      <c r="CG106" s="24" t="n"/>
+      <c r="CH106" s="24" t="n"/>
+      <c r="CI106" s="24" t="n"/>
+      <c r="CJ106" s="24" t="n"/>
+      <c r="CK106" s="24" t="n"/>
+      <c r="CL106" s="24" t="n"/>
+      <c r="CM106" s="24" t="n"/>
+      <c r="CN106" s="24" t="n"/>
+      <c r="CO106" s="24" t="n"/>
+      <c r="CP106" s="24" t="n"/>
+      <c r="CQ106" s="24" t="n"/>
+      <c r="CR106" s="24" t="n"/>
+      <c r="CS106" s="24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="CT106" s="24" t="n"/>
+      <c r="CU106" s="24" t="n"/>
+      <c r="CV106" s="24" t="n"/>
+      <c r="CW106" s="24" t="n"/>
+      <c r="CX106" s="24" t="n"/>
+      <c r="CY106" s="24" t="n"/>
+      <c r="CZ106" s="24" t="n"/>
+      <c r="DA106" s="24" t="n"/>
+      <c r="DB106" s="24" t="n"/>
+      <c r="DC106" s="24" t="n"/>
+      <c r="DD106" s="24" t="n"/>
+      <c r="DE106" s="24" t="n"/>
+      <c r="DF106" s="24" t="n"/>
+      <c r="DG106" s="24" t="n"/>
+      <c r="DH106" s="24" t="n"/>
+      <c r="DI106" s="24" t="n"/>
+      <c r="DJ106" s="24" t="n"/>
+      <c r="DK106" s="24" t="n"/>
+      <c r="DL106" s="24" t="n"/>
+      <c r="DM106" s="24" t="n"/>
+      <c r="DN106" s="24" t="n"/>
+      <c r="DO106" s="24" t="n"/>
+      <c r="DP106" s="24" t="n"/>
+      <c r="DQ106" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "341c7e2b0ea30be66dd305c47452d403a5fa249e98491a2f79156a336a3015bb", "away_team": "KT Wiz", "draw_settlement_value": 0.5, "event_id": "148642", "event_start_utc": "2026-10-11T05:00:00Z", "features": {"away_elo": 1580.7886, "base_tie_rate": 0.02259264, "home_advantage": 20.0, "home_elo": 1535.648797}, "historical_source_observation_times_verified": false, "home_team": "Samsung Lions", "inference_inputs": {"away_id": "KT", "base_tie_rate": 0.02259264, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KT": 1580.7886, "SAMSUNG": 1535.648797}}, "code_sha256": {"features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "SAMSUNG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-11T01:06:46.324600+00:00", "outcome_probabilities": {"away": 0.5240037982249255, "draw": 0.02259264, "home": 0.4534035617750744}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.5353, "home": 0.4647}, "snapshot_hash": "2ac60c4611042d75927eb8c2a2eb75a1dd1836a3e7d286efcf4a0e513d858a37", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="36" customHeight="1">
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t>9a3dfc69ca3444a1</t>
+        </is>
+      </c>
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.217038Z</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T09:30:00Z</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>150824</t>
+        </is>
+      </c>
+      <c r="E107" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F107" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="G107" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="H107" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I107" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J107" s="25" t="n"/>
+      <c r="K107" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L107" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M107" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N107" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O107" s="28" t="n">
+        <v>0.545318</v>
+      </c>
+      <c r="P107" s="28" t="n"/>
+      <c r="Q107" s="28" t="n">
+        <v>-0.09497</v>
+      </c>
+      <c r="R107" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T107" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U107" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V107" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W107" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="X107" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y107" s="25" t="n"/>
+      <c r="Z107" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="AA107" s="28" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AB107" s="28" t="n">
+        <v>-0.000288</v>
+      </c>
+      <c r="AC107" s="30" t="n">
+        <v>0.5618</v>
+      </c>
+      <c r="AD107" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:16:59.472155Z</t>
+        </is>
+      </c>
+      <c r="AE107" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.6400 (market_slug=aec-kbo-sla-kwt-2026-10-12). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF107" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG107" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH107" s="24" t="n"/>
+      <c r="AI107" s="31" t="n"/>
+      <c r="AJ107" s="31" t="n"/>
+      <c r="AK107" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL107" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM107" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN107" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO107" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP107" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AQ107" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AR107" s="24" t="inlineStr">
+        <is>
+          <t>KT Wiz</t>
+        </is>
+      </c>
+      <c r="AS107" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AT107" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AU107" s="24" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="AV107" s="24" t="n"/>
+      <c r="AW107" s="24" t="n"/>
+      <c r="AX107" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY107" s="24" t="n"/>
+      <c r="AZ107" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA107" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BB107" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC107" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD107" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BE107" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF107" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG107" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH107" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.051665Z</t>
+        </is>
+      </c>
+      <c r="BI107" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ107" s="25" t="n"/>
+      <c r="BK107" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL107" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM107" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN107" s="28" t="n"/>
+      <c r="BO107" s="28" t="n"/>
+      <c r="BP107" s="25" t="n"/>
+      <c r="BQ107" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BR107" s="28" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="BS107" s="28" t="n"/>
+      <c r="BT107" s="28" t="n"/>
+      <c r="BU107" s="25" t="n"/>
+      <c r="BV107" s="29" t="n"/>
+      <c r="BW107" s="24" t="n"/>
+      <c r="BX107" s="30" t="n"/>
+      <c r="BY107" s="27" t="n"/>
+      <c r="BZ107" s="24" t="n"/>
+      <c r="CA107" s="31" t="n"/>
+      <c r="CB107" s="24" t="n"/>
+      <c r="CC107" s="24" t="n"/>
+      <c r="CD107" s="24" t="n"/>
+      <c r="CE107" s="24" t="n"/>
+      <c r="CF107" s="24" t="n"/>
+      <c r="CG107" s="24" t="n"/>
+      <c r="CH107" s="24" t="n"/>
+      <c r="CI107" s="24" t="n"/>
+      <c r="CJ107" s="24" t="n"/>
+      <c r="CK107" s="24" t="n"/>
+      <c r="CL107" s="24" t="n"/>
+      <c r="CM107" s="24" t="n"/>
+      <c r="CN107" s="24" t="n"/>
+      <c r="CO107" s="24" t="n"/>
+      <c r="CP107" s="24" t="n"/>
+      <c r="CQ107" s="24" t="n"/>
+      <c r="CR107" s="24" t="n"/>
+      <c r="CS107" s="24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="CT107" s="24" t="n"/>
+      <c r="CU107" s="24" t="n"/>
+      <c r="CV107" s="24" t="n"/>
+      <c r="CW107" s="24" t="n"/>
+      <c r="CX107" s="24" t="n"/>
+      <c r="CY107" s="24" t="n"/>
+      <c r="CZ107" s="24" t="n"/>
+      <c r="DA107" s="24" t="n"/>
+      <c r="DB107" s="24" t="n"/>
+      <c r="DC107" s="24" t="n"/>
+      <c r="DD107" s="24" t="n"/>
+      <c r="DE107" s="24" t="n"/>
+      <c r="DF107" s="24" t="n"/>
+      <c r="DG107" s="24" t="n"/>
+      <c r="DH107" s="24" t="n"/>
+      <c r="DI107" s="24" t="n"/>
+      <c r="DJ107" s="24" t="n"/>
+      <c r="DK107" s="24" t="n"/>
+      <c r="DL107" s="24" t="n"/>
+      <c r="DM107" s="24" t="n"/>
+      <c r="DN107" s="24" t="n"/>
+      <c r="DO107" s="24" t="n"/>
+      <c r="DP107" s="24" t="n"/>
+      <c r="DQ107" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b", "away_team": "KT Wiz", "draw_settlement_value": 0.5, "event_id": "150824", "event_start_utc": "2026-10-12T09:30:00Z", "features": {"away_elo": 1584.177002, "base_tie_rate": 0.02258642, "home_advantage": 20.0, "home_elo": 1531.866464}, "historical_source_observation_times_verified": false, "home_team": "Samsung Lions", "inference_inputs": {"away_id": "KT", "base_tie_rate": 0.02258642, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KT": 1584.177002, "SAMSUNG": 1531.866464}}, "code_sha256": {"features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "SAMSUNG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-12T05:39:16.914450+00:00", "outcome_probabilities": {"away": 0.5340245869223879, "draw": 0.02258642, "home": 0.4433889930776122}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.545318, "home": 0.454682}, "snapshot_hash": "414f5b656cf89e6e627a764df1550d638c17439ddebd33e82e621ef327a6e6ed", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="36" customHeight="1">
+      <c r="A108" s="24" t="inlineStr">
+        <is>
+          <t>1f72099515a84baf</t>
+        </is>
+      </c>
+      <c r="B108" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.217038Z</t>
+        </is>
+      </c>
+      <c r="C108" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T09:30:00Z</t>
+        </is>
+      </c>
+      <c r="D108" s="24" t="inlineStr">
+        <is>
+          <t>150825</t>
+        </is>
+      </c>
+      <c r="E108" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F108" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="G108" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="H108" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I108" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J108" s="25" t="n"/>
+      <c r="K108" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L108" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="M108" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="N108" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="O108" s="28" t="n">
+        <v>0.576893</v>
+      </c>
+      <c r="P108" s="28" t="n"/>
+      <c r="Q108" s="28" t="n">
+        <v>0.116064</v>
+      </c>
+      <c r="R108" s="26" t="n">
+        <v>78</v>
+      </c>
+      <c r="S108" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T108" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U108" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V108" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W108" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X108" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y108" s="25" t="n"/>
+      <c r="Z108" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="AA108" s="28" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AB108" s="28" t="n">
+        <v>-0.000829</v>
+      </c>
+      <c r="AC108" s="30" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AD108" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:17:02.221787Z</t>
+        </is>
+      </c>
+      <c r="AE108" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.4600 (market_slug=aec-kbo-dbo-lgo-2026-10-12). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF108" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG108" s="24" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+      <c r="AH108" s="24" t="n"/>
+      <c r="AI108" s="31" t="n"/>
+      <c r="AJ108" s="31" t="n"/>
+      <c r="AK108" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL108" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM108" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN108" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO108" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP108" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AQ108" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AR108" s="24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="AS108" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AT108" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AU108" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AV108" s="24" t="n"/>
+      <c r="AW108" s="24" t="n"/>
+      <c r="AX108" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY108" s="24" t="n"/>
+      <c r="AZ108" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA108" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BB108" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC108" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD108" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BE108" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF108" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG108" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH108" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.127133Z</t>
+        </is>
+      </c>
+      <c r="BI108" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ108" s="25" t="n"/>
+      <c r="BK108" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="BL108" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="BM108" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="BN108" s="28" t="n"/>
+      <c r="BO108" s="28" t="n"/>
+      <c r="BP108" s="25" t="n"/>
+      <c r="BQ108" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="BR108" s="28" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="BS108" s="28" t="n"/>
+      <c r="BT108" s="28" t="n"/>
+      <c r="BU108" s="25" t="n"/>
+      <c r="BV108" s="29" t="n"/>
+      <c r="BW108" s="24" t="n"/>
+      <c r="BX108" s="30" t="n"/>
+      <c r="BY108" s="27" t="n"/>
+      <c r="BZ108" s="24" t="n"/>
+      <c r="CA108" s="31" t="n"/>
+      <c r="CB108" s="24" t="n"/>
+      <c r="CC108" s="24" t="n"/>
+      <c r="CD108" s="24" t="n"/>
+      <c r="CE108" s="24" t="n"/>
+      <c r="CF108" s="24" t="n"/>
+      <c r="CG108" s="24" t="n"/>
+      <c r="CH108" s="24" t="n"/>
+      <c r="CI108" s="24" t="n"/>
+      <c r="CJ108" s="24" t="n"/>
+      <c r="CK108" s="24" t="n"/>
+      <c r="CL108" s="24" t="n"/>
+      <c r="CM108" s="24" t="n"/>
+      <c r="CN108" s="24" t="n"/>
+      <c r="CO108" s="24" t="n"/>
+      <c r="CP108" s="24" t="n"/>
+      <c r="CQ108" s="24" t="n"/>
+      <c r="CR108" s="24" t="n"/>
+      <c r="CS108" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT108" s="24" t="n"/>
+      <c r="CU108" s="24" t="n"/>
+      <c r="CV108" s="24" t="n"/>
+      <c r="CW108" s="24" t="n"/>
+      <c r="CX108" s="24" t="n"/>
+      <c r="CY108" s="24" t="n"/>
+      <c r="CZ108" s="24" t="n"/>
+      <c r="DA108" s="24" t="n"/>
+      <c r="DB108" s="24" t="n"/>
+      <c r="DC108" s="24" t="n"/>
+      <c r="DD108" s="24" t="n"/>
+      <c r="DE108" s="24" t="n"/>
+      <c r="DF108" s="24" t="n"/>
+      <c r="DG108" s="24" t="n"/>
+      <c r="DH108" s="24" t="n"/>
+      <c r="DI108" s="24" t="n"/>
+      <c r="DJ108" s="24" t="n"/>
+      <c r="DK108" s="24" t="n"/>
+      <c r="DL108" s="24" t="n"/>
+      <c r="DM108" s="24" t="n"/>
+      <c r="DN108" s="24" t="n"/>
+      <c r="DO108" s="24" t="n"/>
+      <c r="DP108" s="24" t="n"/>
+      <c r="DQ108" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b", "away_team": "Lotte Giants", "draw_settlement_value": 0.5, "event_id": "150825", "event_start_utc": "2026-10-12T09:30:00Z", "features": {"away_elo": 1484.286182, "base_tie_rate": 0.02258642, "home_advantage": 20.0, "home_elo": 1519.40969}, "historical_source_observation_times_verified": false, "home_team": "Doosan Bears", "inference_inputs": {"away_id": "LOTTE", "base_tie_rate": 0.02258642, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"DOOSAN": 1519.40969, "LOTTE": 1484.286182}}, "code_sha256": {"features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "DOOSAN", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-12T05:39:16.914450+00:00", "outcome_probabilities": {"away": 0.4118135618586591, "draw": 0.02258642, "home": 0.5656000181413409}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.423107, "home": 0.576893}, "snapshot_hash": "a3c933a5546196d889ef02b4634a48b6cafaa117eb9a807e14f0674e3fa214b1", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="36" customHeight="1">
+      <c r="A109" s="24" t="inlineStr">
+        <is>
+          <t>19078efa028f406c</t>
+        </is>
+      </c>
+      <c r="B109" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.217038Z</t>
+        </is>
+      </c>
+      <c r="C109" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T09:30:00Z</t>
+        </is>
+      </c>
+      <c r="D109" s="24" t="inlineStr">
+        <is>
+          <t>150826</t>
+        </is>
+      </c>
+      <c r="E109" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F109" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="G109" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="H109" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I109" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J109" s="25" t="n"/>
+      <c r="K109" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L109" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M109" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N109" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O109" s="28" t="n">
+        <v>0.555504</v>
+      </c>
+      <c r="P109" s="28" t="n"/>
+      <c r="Q109" s="28" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="R109" s="26" t="n">
+        <v>43</v>
+      </c>
+      <c r="S109" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T109" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U109" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V109" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W109" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="X109" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y109" s="25" t="n"/>
+      <c r="Z109" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="AA109" s="28" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AB109" s="28" t="n">
+        <v>0.000196</v>
+      </c>
+      <c r="AC109" s="30" t="n">
+        <v>0.9615</v>
+      </c>
+      <c r="AD109" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:17:05.324741Z</t>
+        </is>
+      </c>
+      <c r="AE109" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.5100 (market_slug=aec-kbo-kti-ltg-2026-10-12). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF109" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG109" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH109" s="24" t="n"/>
+      <c r="AI109" s="31" t="n"/>
+      <c r="AJ109" s="31" t="n"/>
+      <c r="AK109" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL109" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM109" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN109" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO109" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP109" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AQ109" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AR109" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AS109" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AT109" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AU109" s="24" t="inlineStr">
+        <is>
+          <t>Kia Tigers</t>
+        </is>
+      </c>
+      <c r="AV109" s="24" t="n"/>
+      <c r="AW109" s="24" t="n"/>
+      <c r="AX109" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY109" s="24" t="n"/>
+      <c r="AZ109" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA109" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BB109" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC109" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD109" s="24" t="inlineStr">
+        <is>
+          <t>f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b</t>
+        </is>
+      </c>
+      <c r="BE109" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF109" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG109" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH109" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:39:17.217038Z</t>
+        </is>
+      </c>
+      <c r="BI109" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ109" s="25" t="n"/>
+      <c r="BK109" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL109" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM109" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN109" s="28" t="n"/>
+      <c r="BO109" s="28" t="n"/>
+      <c r="BP109" s="25" t="n"/>
+      <c r="BQ109" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BR109" s="28" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="BS109" s="28" t="n"/>
+      <c r="BT109" s="28" t="n"/>
+      <c r="BU109" s="25" t="n"/>
+      <c r="BV109" s="29" t="n"/>
+      <c r="BW109" s="24" t="n"/>
+      <c r="BX109" s="30" t="n"/>
+      <c r="BY109" s="27" t="n"/>
+      <c r="BZ109" s="24" t="n"/>
+      <c r="CA109" s="31" t="n"/>
+      <c r="CB109" s="24" t="n"/>
+      <c r="CC109" s="24" t="n"/>
+      <c r="CD109" s="24" t="n"/>
+      <c r="CE109" s="24" t="n"/>
+      <c r="CF109" s="24" t="n"/>
+      <c r="CG109" s="24" t="n"/>
+      <c r="CH109" s="24" t="n"/>
+      <c r="CI109" s="24" t="n"/>
+      <c r="CJ109" s="24" t="n"/>
+      <c r="CK109" s="24" t="n"/>
+      <c r="CL109" s="24" t="n"/>
+      <c r="CM109" s="24" t="n"/>
+      <c r="CN109" s="24" t="n"/>
+      <c r="CO109" s="24" t="n"/>
+      <c r="CP109" s="24" t="n"/>
+      <c r="CQ109" s="24" t="n"/>
+      <c r="CR109" s="24" t="n"/>
+      <c r="CS109" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT109" s="24" t="n"/>
+      <c r="CU109" s="24" t="n"/>
+      <c r="CV109" s="24" t="n"/>
+      <c r="CW109" s="24" t="n"/>
+      <c r="CX109" s="24" t="n"/>
+      <c r="CY109" s="24" t="n"/>
+      <c r="CZ109" s="24" t="n"/>
+      <c r="DA109" s="24" t="n"/>
+      <c r="DB109" s="24" t="n"/>
+      <c r="DC109" s="24" t="n"/>
+      <c r="DD109" s="24" t="n"/>
+      <c r="DE109" s="24" t="n"/>
+      <c r="DF109" s="24" t="n"/>
+      <c r="DG109" s="24" t="n"/>
+      <c r="DH109" s="24" t="n"/>
+      <c r="DI109" s="24" t="n"/>
+      <c r="DJ109" s="24" t="n"/>
+      <c r="DK109" s="24" t="n"/>
+      <c r="DL109" s="24" t="n"/>
+      <c r="DM109" s="24" t="n"/>
+      <c r="DN109" s="24" t="n"/>
+      <c r="DO109" s="24" t="n"/>
+      <c r="DP109" s="24" t="n"/>
+      <c r="DQ109" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "f828956be898ea82909cc2c95471f23915163bd39f9e25da1a377dad461ebb9b", "away_team": "LG Twins", "draw_settlement_value": 0.5, "event_id": "150826", "event_start_utc": "2026-10-12T09:30:00Z", "features": {"away_elo": 1510.493341, "base_tie_rate": 0.02258642, "home_advantage": 20.0, "home_elo": 1530.123769}, "historical_source_observation_times_verified": false, "home_team": "Kia Tigers", "inference_inputs": {"away_id": "LG", "base_tie_rate": 0.02258642, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"KIA": 1530.123769, "LG": 1510.493341}}, "code_sha256": {"features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "KIA", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-12T05:39:16.914450+00:00", "outcome_probabilities": {"away": 0.433202697383019, "draw": 0.02258642, "home": 0.544210882616981}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.444496, "home": 0.555504}, "snapshot_hash": "1abf9f56510029fa32df9cc61fe09feb73cb594b4d6317de7c8a57cac5a0dd14", "sport": "KBO"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="36" customHeight="1">
+      <c r="A110" s="24" t="inlineStr">
+        <is>
+          <t>044ae5cf87ae450a</t>
+        </is>
+      </c>
+      <c r="B110" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-13T22:28:51.817150Z</t>
+        </is>
+      </c>
+      <c r="C110" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T09:30:00Z</t>
+        </is>
+      </c>
+      <c r="D110" s="24" t="inlineStr">
+        <is>
+          <t>156781</t>
+        </is>
+      </c>
+      <c r="E110" s="24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="F110" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="G110" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="H110" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I110" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J110" s="25" t="n"/>
+      <c r="K110" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L110" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="M110" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="N110" s="28" t="n">
+        <v>0.469484</v>
+      </c>
+      <c r="O110" s="28" t="n">
+        <v>0.517455</v>
+      </c>
+      <c r="P110" s="28" t="n"/>
+      <c r="Q110" s="28" t="n">
+        <v>0.047971</v>
+      </c>
+      <c r="R110" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="S110" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T110" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="U110" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V110" s="24" t="n"/>
+      <c r="W110" s="26" t="n"/>
+      <c r="X110" s="26" t="n"/>
+      <c r="Y110" s="25" t="n"/>
+      <c r="Z110" s="26" t="n"/>
+      <c r="AA110" s="28" t="n"/>
+      <c r="AB110" s="28" t="n"/>
+      <c r="AC110" s="30" t="n"/>
+      <c r="AD110" s="24" t="n"/>
+      <c r="AE110" s="31" t="inlineStr">
+        <is>
+          <t>Tie-aware Elo baseline; executable ask 0.4700 (market_slug=aec-kbo-ltg-dbo-2026-10-14). Tie probability=0.0226.</t>
+        </is>
+      </c>
+      <c r="AF110" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted international baseball baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG110" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH110" s="24" t="n"/>
+      <c r="AI110" s="31" t="n"/>
+      <c r="AJ110" s="31" t="n"/>
+      <c r="AK110" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL110" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM110" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN110" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO110" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP110" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AQ110" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AR110" s="24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="AS110" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AT110" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AU110" s="24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="AV110" s="24" t="n"/>
+      <c r="AW110" s="24" t="n"/>
+      <c r="AX110" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY110" s="24" t="n"/>
+      <c r="AZ110" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA110" s="24" t="inlineStr">
+        <is>
+          <t>a8edff19ea33759e916156f0340eeb6b44b7dd1ede0ca462f6ded28493f70ba6</t>
+        </is>
+      </c>
+      <c r="BB110" s="24" t="inlineStr">
+        <is>
+          <t>tie_aware_elo</t>
+        </is>
+      </c>
+      <c r="BC110" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BD110" s="24" t="inlineStr">
+        <is>
+          <t>a8edff19ea33759e916156f0340eeb6b44b7dd1ede0ca462f6ded28493f70ba6</t>
+        </is>
+      </c>
+      <c r="BE110" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF110" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG110" s="24" t="inlineStr">
+        <is>
+          <t>kbo-tie-aware-elo-v2</t>
+        </is>
+      </c>
+      <c r="BH110" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-13T22:28:51.817150Z</t>
+        </is>
+      </c>
+      <c r="BI110" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ110" s="25" t="n"/>
+      <c r="BK110" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="BL110" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="BM110" s="28" t="n">
+        <v>0.469484</v>
+      </c>
+      <c r="BN110" s="28" t="n"/>
+      <c r="BO110" s="28" t="n"/>
+      <c r="BP110" s="25" t="n"/>
+      <c r="BQ110" s="27" t="n"/>
+      <c r="BR110" s="28" t="n"/>
+      <c r="BS110" s="28" t="n"/>
+      <c r="BT110" s="28" t="n"/>
+      <c r="BU110" s="25" t="n"/>
+      <c r="BV110" s="29" t="n"/>
+      <c r="BW110" s="24" t="n"/>
+      <c r="BX110" s="30" t="n"/>
+      <c r="BY110" s="27" t="n"/>
+      <c r="BZ110" s="24" t="n"/>
+      <c r="CA110" s="31" t="n"/>
+      <c r="CB110" s="24" t="n"/>
+      <c r="CC110" s="24" t="n"/>
+      <c r="CD110" s="24" t="n"/>
+      <c r="CE110" s="24" t="n"/>
+      <c r="CF110" s="24" t="n"/>
+      <c r="CG110" s="24" t="n"/>
+      <c r="CH110" s="24" t="n"/>
+      <c r="CI110" s="24" t="n"/>
+      <c r="CJ110" s="24" t="n"/>
+      <c r="CK110" s="24" t="n"/>
+      <c r="CL110" s="24" t="n"/>
+      <c r="CM110" s="24" t="n"/>
+      <c r="CN110" s="24" t="n"/>
+      <c r="CO110" s="24" t="n"/>
+      <c r="CP110" s="24" t="n"/>
+      <c r="CQ110" s="24" t="n"/>
+      <c r="CR110" s="24" t="n"/>
+      <c r="CS110" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT110" s="24" t="n"/>
+      <c r="CU110" s="24" t="n"/>
+      <c r="CV110" s="24" t="n"/>
+      <c r="CW110" s="24" t="n"/>
+      <c r="CX110" s="24" t="n"/>
+      <c r="CY110" s="24" t="n"/>
+      <c r="CZ110" s="24" t="n"/>
+      <c r="DA110" s="24" t="n"/>
+      <c r="DB110" s="24" t="n"/>
+      <c r="DC110" s="24" t="n"/>
+      <c r="DD110" s="24" t="n"/>
+      <c r="DE110" s="24" t="n"/>
+      <c r="DF110" s="24" t="n"/>
+      <c r="DG110" s="24" t="n"/>
+      <c r="DH110" s="24" t="n"/>
+      <c r="DI110" s="24" t="n"/>
+      <c r="DJ110" s="24" t="n"/>
+      <c r="DK110" s="24" t="n"/>
+      <c r="DL110" s="24" t="n"/>
+      <c r="DM110" s="24" t="n"/>
+      <c r="DN110" s="24" t="n"/>
+      <c r="DO110" s="24" t="n"/>
+      <c r="DP110" s="24" t="n"/>
+      <c r="DQ110" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "a8edff19ea33759e916156f0340eeb6b44b7dd1ede0ca462f6ded28493f70ba6", "away_team": "Doosan Bears", "draw_settlement_value": 0.5, "event_id": "156781", "event_start_utc": "2026-10-14T09:30:00Z", "features": {"away_elo": 1514.491213, "base_tie_rate": 0.02257709, "home_advantage": 20.0, "home_elo": 1506.905724}, "historical_source_observation_times_verified": false, "home_team": "LG Twins", "inference_inputs": {"away_id": "DOOSAN", "base_tie_rate": 0.02257709, "book_state": {"_games_played": null, "_last_active": null, "decay_rate": 0.001, "home_advantage": 20.0, "k": 8.0, "margin_weight": 0.0, "ratings": {"DOOSAN": 1514.491213, "LG": 1506.905724}}, "code_sha256": {"features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872", "international_baseball.py": "fe583791ae4febdb6b477e979042a87e118f547c292d23a5c6651da0218cc4e4"}, "home_id": "LG", "tie_method": "flat"}, "market_type": "moneyline", "model_version": "kbo-tie-aware-elo-v2", "observed_at_utc": "2026-10-13T22:28:51.165973+00:00", "outcome_probabilities": {"away": 0.4712563260098324, "draw": 0.02257709, "home": 0.5061665839901677}, "replay_scope": "Exact Elo and tie model; logged value is expected contract settlement, not outright win probability.", "schema": "international-elo-replay-v1", "settlement_values": {"away": 0.482545, "home": 0.517455}, "snapshot_hash": "f882f37433c0065bdadd8cf508c7d60dfe772b18ee84ebf7e3a79569e5493f65", "sport": "KBO"}</t>
         </is>
       </c>
     </row>

</xml_diff>